<commit_message>
Fix broken menu links to StructureDefinition-FRLMHeaderDocument/FRLMCorpsDocument
Le menu pointait vers des noms de fichiers en kebab-case (fr-lm-header-document,
fr-lm-corps-document) qui n'ont jamais correspondu aux Id FSH réels
(FRLMHeaderDocument, FRLMCorpsDocument). Ces liens cassés apparaissaient dans
le nav de chaque page générée, gonflant le compteur de Build Errors du QA
(des milliers d'occurrences pour 2 liens cassés à la base). f4092b4968aa99d95d457845feba57ab945d72af
</commit_message>
<xml_diff>
--- a/fix-target-codes-and-display/ig/StructureDefinition-FRLMAdvanceDirective.xlsx
+++ b/fix-target-codes-and-display/ig/StructureDefinition-FRLMAdvanceDirective.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-20T08:53:12+00:00</t>
+    <t>2026-08-20T15:08:45+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -466,7 +466,7 @@
     <t>jdv-type-directive-anticipee-cisis (1.2.250.1.213.1.1.5.136)</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-type-directive-anticipee-cisis|20260619134043</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-type-directive-anticipee-cisis|20260716085853</t>
   </si>
   <si>
     <t>FRLMAdvanceDirective.value</t>

</xml_diff>